<commit_message>
Add Highlight function for each action
</commit_message>
<xml_diff>
--- a/data/Conferences.xlsx
+++ b/data/Conferences.xlsx
@@ -51,7 +51,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +61,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.3999450666829432"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF99"/>
+        <bgColor rgb="00FFFF99"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,7 +87,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -111,6 +117,25 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -484,53 +509,53 @@
       </c>
     </row>
     <row r="2" ht="33" customHeight="1" s="8">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>系统</t>
         </is>
       </c>
-      <c r="B2" s="0" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>PPoPP</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>ACM SIGPLAN Symposium on Principles &amp; Practice of Parallel Programming</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>ACM</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>Salt Lake City, (Utah), USA</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="15" t="inlineStr">
         <is>
           <t>03.20-03.24</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H2" s="9" t="inlineStr">
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H2" s="16" t="inlineStr">
         <is>
           <t>https://ppopp27.sigplan.org/</t>
         </is>
       </c>
-      <c r="I2" s="0" t="inlineStr"/>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>需要人工核实官网（未配置搜索API做兜底）</t>
-        </is>
-      </c>
-      <c r="K2" s="7" t="n"/>
+      <c r="I2" s="11" t="inlineStr"/>
+      <c r="J2" s="17" t="inlineStr">
+        <is>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
+        </is>
+      </c>
+      <c r="K2" s="17" t="n"/>
     </row>
     <row r="3" ht="48.75" customHeight="1" s="8">
       <c r="A3" s="0" t="inlineStr">
@@ -3346,7 +3371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3376,6 +3401,60 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>AAAI</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>FAKE_TEST_VALUE</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E2" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-22 21:43 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PPoPP</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>WRONG_DDL_TEST</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-07-22 21:46 UTC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: weekly deadline update
</commit_message>
<xml_diff>
--- a/data/Conferences.xlsx
+++ b/data/Conferences.xlsx
@@ -509,101 +509,102 @@
       </c>
     </row>
     <row r="2" ht="33" customHeight="1" s="8">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>系统</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>PPoPP</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>ACM SIGPLAN Symposium on Principles &amp; Practice of Parallel Programming</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>ACM</t>
         </is>
       </c>
-      <c r="E2" s="15" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Salt Lake City, (Utah), USA</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>03.20-03.24</t>
         </is>
       </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H2" s="16" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>https://ppopp27.sigplan.org/</t>
         </is>
       </c>
-      <c r="I2" s="11" t="inlineStr"/>
-      <c r="J2" s="17" t="inlineStr">
-        <is>
-          <t>需要人工核实官网（未配置搜索API做兜底）</t>
-        </is>
-      </c>
-      <c r="K2" s="17" t="n"/>
+      <c r="I2" s="0" t="inlineStr"/>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
+        </is>
+      </c>
+      <c r="K2" s="7" t="n"/>
     </row>
     <row r="3" ht="48.75" customHeight="1" s="8">
-      <c r="A3" s="0" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>软工</t>
         </is>
       </c>
-      <c r="B3" s="0" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>FSE/ESEC</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>ACM Joint European Software Engineering Conference and Symposium on the Foundations of Software Engineering</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>ACM</t>
         </is>
       </c>
-      <c r="E3" s="0" t="inlineStr">
-        <is>
-          <t>Shenzhen, China</t>
-        </is>
-      </c>
-      <c r="F3" s="0" t="inlineStr">
-        <is>
-          <t>07.12-07.16</t>
-        </is>
-      </c>
-      <c r="G3" s="0" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="inlineStr">
         <is>
           <t>https://conf.researchr.org/home/fse-2027</t>
         </is>
       </c>
-      <c r="I3" s="0" t="inlineStr"/>
-      <c r="J3" s="0" t="inlineStr">
-        <is>
-          <t>需要人工核实官网（未配置搜索API做兜底）</t>
-        </is>
-      </c>
+      <c r="I3" s="11" t="inlineStr"/>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="n"/>
     </row>
     <row r="4" ht="26.5" customHeight="1" s="8">
       <c r="A4" s="0" t="inlineStr">
@@ -1018,48 +1019,53 @@
       </c>
     </row>
     <row r="13" ht="26.5" customHeight="1" s="8">
-      <c r="A13" s="0" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>网络</t>
         </is>
       </c>
-      <c r="B13" s="0" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>MobiCom</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>ACM International Conference on Mobile Computing and Networking</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>ACM</t>
         </is>
       </c>
-      <c r="E13" s="0" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F13" s="0" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G13" s="0" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="0" t="inlineStr"/>
-      <c r="J13" s="0" t="inlineStr">
-        <is>
-          <t>需要人工核实官网（未配置搜索API做兜底）</t>
-        </is>
-      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>10.18-10.22</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sigmobile.org/mobicom/2027/</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr"/>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
+        </is>
+      </c>
+      <c r="K13" s="13" t="n"/>
     </row>
     <row r="14" ht="26.5" customHeight="1" s="8">
       <c r="A14" s="0" t="inlineStr">
@@ -3325,31 +3331,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId32"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.7480314960629921" right="0.7480314960629921" top="0.984251968503937" bottom="0.984251968503937" header="0.5118110236220472" footer="0.5118110236220472"/>
@@ -3429,27 +3436,27 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>PPoPP</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>Workshop Deadline</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>WRONG_DDL_TEST</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
         <is>
           <t>2026-07-22 21:46 UTC</t>
         </is>

</xml_diff>

<commit_message>
Fix Brave Search secret name mismatch and FSE name-collision bug
- Workflow referenced secrets.BRAVE_SEARCH_API_KEY but the configured
  secret is named BRAVE_SEARCH_APIKEY, so the key silently resolved to
  empty and Brave Search fallback never ran
- ccfddl has two unrelated conferences both titled "FSE" (Foundations of
  Software Engineering vs Fast Software Encryption); dict-keyed lookup by
  slug alone let filesystem traversal order pick the wrong one depending
  on OS, which produced correct results locally but wrong ones on the
  Linux Actions runner. Lookup is now keyed by (slug, category) and
  ambiguous acronyms must be disambiguated explicitly in ALIASES
</commit_message>
<xml_diff>
--- a/data/Conferences.xlsx
+++ b/data/Conferences.xlsx
@@ -580,12 +580,12 @@
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Shenzhen, China</t>
         </is>
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>07.12-07.16</t>
         </is>
       </c>
       <c r="G3" s="11" t="inlineStr">
@@ -1019,53 +1019,52 @@
       </c>
     </row>
     <row r="13" ht="26.5" customHeight="1" s="8">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>网络</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>MobiCom</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>ACM International Conference on Mobile Computing and Networking</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>ACM</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
         <is>
           <t>10.18-10.22</t>
         </is>
       </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
         <is>
           <t>https://www.sigmobile.org/mobicom/2027/</t>
         </is>
       </c>
-      <c r="I13" s="11" t="inlineStr"/>
-      <c r="J13" s="11" t="inlineStr">
-        <is>
-          <t>需要人工核实官网（未配置搜索API做兜底）</t>
-        </is>
-      </c>
-      <c r="K13" s="13" t="n"/>
+      <c r="I13" s="0" t="inlineStr"/>
+      <c r="J13" s="0" t="inlineStr">
+        <is>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="26.5" customHeight="1" s="8">
       <c r="A14" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Disable Brave Search fallback for now, clean up bad results it produced
2027 workshop info mostly hasn't been published yet, so search fallback
was mostly returning false positives (stale pages, unrelated pages, one
generic page matched across a dozen unrelated conferences with the same
bogus 2026.09.04 date). Commented out the secret env var in the workflow
so it's easy to re-enable later once conferences actually start
publishing workshop CFPs; re-ran the checker without it to restore
accurate TBD/confirmed state.
</commit_message>
<xml_diff>
--- a/data/Conferences.xlsx
+++ b/data/Conferences.xlsx
@@ -541,7 +541,7 @@
       </c>
       <c r="G2" s="15" t="inlineStr">
         <is>
-          <t>2026.07.24</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H2" s="16" t="inlineStr">
@@ -549,14 +549,10 @@
           <t>https://ppopp27.sigplan.org/</t>
         </is>
       </c>
-      <c r="I2" s="16" t="inlineStr">
-        <is>
-          <t>https://popl27.sigplan.org/track/POPL-2027-workshops-and-co-located-events</t>
-        </is>
-      </c>
+      <c r="I2" s="16" t="inlineStr"/>
       <c r="J2" s="17" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K2" s="17" t="n"/>
@@ -594,7 +590,7 @@
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
-          <t>2027.03.05</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H3" s="14" t="inlineStr">
@@ -602,14 +598,10 @@
           <t>https://conf.researchr.org/home/fse-2027</t>
         </is>
       </c>
-      <c r="I3" s="16" t="inlineStr">
-        <is>
-          <t>https://conf.researchr.org/home/fse-2027</t>
-        </is>
-      </c>
+      <c r="I3" s="16" t="inlineStr"/>
       <c r="J3" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K3" s="13" t="n"/>
@@ -647,7 +639,7 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>2026.05.19</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H4" s="14" t="inlineStr">
@@ -655,14 +647,10 @@
           <t>https://icde2027.github.io/</t>
         </is>
       </c>
-      <c r="I4" s="16" t="inlineStr">
-        <is>
-          <t>https://icde2027.github.io/</t>
-        </is>
-      </c>
+      <c r="I4" s="16" t="inlineStr"/>
       <c r="J4" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K4" s="13" t="n"/>
@@ -711,7 +699,7 @@
       <c r="I5" s="0" t="inlineStr"/>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t>抓取+搜索兜底均未找到，需人工核实</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -748,18 +736,14 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>2026.09.28</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H6" s="12" t="inlineStr"/>
-      <c r="I6" s="16" t="inlineStr">
-        <is>
-          <t>https://chi2027.acm.org/authors/workshops/</t>
-        </is>
-      </c>
+      <c r="I6" s="16" t="inlineStr"/>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K6" s="13" t="n"/>
@@ -797,18 +781,14 @@
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>2026.08.28</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H7" s="12" t="inlineStr"/>
-      <c r="I7" s="16" t="inlineStr">
-        <is>
-          <t>https://sc26.supercomputing.org/all-dates-deadlines/</t>
-        </is>
-      </c>
+      <c r="I7" s="16" t="inlineStr"/>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K7" s="13" t="n"/>
@@ -857,7 +837,7 @@
       <c r="I8" s="0" t="inlineStr"/>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t>抓取+搜索兜底均未找到，需人工核实</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -901,7 +881,7 @@
       <c r="I9" s="0" t="inlineStr"/>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t>抓取+搜索兜底均未找到，需人工核实</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -945,7 +925,7 @@
       <c r="I10" s="0" t="inlineStr"/>
       <c r="J10" s="0" t="inlineStr">
         <is>
-          <t>抓取+搜索兜底均未找到，需人工核实</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -982,7 +962,7 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>2026.08.21</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H11" s="14" t="inlineStr">
@@ -990,14 +970,10 @@
           <t>https://2027.eurosys.org/</t>
         </is>
       </c>
-      <c r="I11" s="16" t="inlineStr">
-        <is>
-          <t>https://2027.eurosys.org/cfp.html</t>
-        </is>
-      </c>
+      <c r="I11" s="16" t="inlineStr"/>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K11" s="13" t="n"/>
@@ -1039,14 +1015,10 @@
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>https://www.sigcomm.org/news</t>
-        </is>
-      </c>
+      <c r="I12" s="9" t="inlineStr"/>
       <c r="J12" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 June 14th, 2024 和会议年份 2027 对不上），需人工核实：https://www.sigcomm.org/news</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1055,7 @@
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H13" s="14" t="inlineStr">
@@ -1091,14 +1063,10 @@
           <t>https://www.sigmobile.org/mobicom/2027/</t>
         </is>
       </c>
-      <c r="I13" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I13" s="16" t="inlineStr"/>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K13" s="13" t="n"/>
@@ -1136,7 +1104,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>2026.11.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H14" s="14" t="inlineStr">
@@ -1144,14 +1112,10 @@
           <t>https://infocom2027.ieee-infocom.org/</t>
         </is>
       </c>
-      <c r="I14" s="16" t="inlineStr">
-        <is>
-          <t>https://mpc-deadlines.github.io/</t>
-        </is>
-      </c>
+      <c r="I14" s="16" t="inlineStr"/>
       <c r="J14" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K14" s="13" t="n"/>
@@ -1200,7 +1164,7 @@
       <c r="I15" s="0" t="inlineStr"/>
       <c r="J15" s="0" t="inlineStr">
         <is>
-          <t>抓取+搜索兜底均未找到，需人工核实</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -1241,14 +1205,10 @@
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>http://www.wikicfp.com/cfp/program?id=399</t>
-        </is>
-      </c>
+      <c r="I16" s="9" t="inlineStr"/>
       <c r="J16" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 4 May 2023 和会议年份 2027 对不上），需人工核实：http://www.wikicfp.com/cfp/program?id=399</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1245,7 @@
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>2026.09.17</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H17" s="14" t="inlineStr">
@@ -1293,14 +1253,10 @@
           <t>https://eurocrypt.iacr.org/2027/</t>
         </is>
       </c>
-      <c r="I17" s="16" t="inlineStr">
-        <is>
-          <t>https://eurocrypt.iacr.org/2027/callforpapers.php</t>
-        </is>
-      </c>
+      <c r="I17" s="16" t="inlineStr"/>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K17" s="13" t="n"/>
@@ -1346,14 +1302,10 @@
           <t>https://sp2027.ieee-security.org/index.html</t>
         </is>
       </c>
-      <c r="I18" s="9" t="inlineStr">
-        <is>
-          <t>https://signalprocessingsociety.org/events/call-proposals-ssp-2027-2027-ieee-statistical-signal-processing-workshop</t>
-        </is>
-      </c>
+      <c r="I18" s="9" t="inlineStr"/>
       <c r="J18" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 27 November 2024 和会议年份 2027 对不上），需人工核实：https://signalprocessingsociety.org/events/call-proposals-ssp-2027-2027-ieee-statistical-signal-processing-workshop</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -1390,18 +1342,14 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>2026.07.26</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H19" s="12" t="inlineStr"/>
-      <c r="I19" s="16" t="inlineStr">
-        <is>
-          <t>https://www.iacr.org/events/eventsbysubmission.php4</t>
-        </is>
-      </c>
+      <c r="I19" s="16" t="inlineStr"/>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K19" s="13" t="n"/>
@@ -1450,7 +1398,7 @@
       <c r="I20" s="0" t="inlineStr"/>
       <c r="J20" s="0" t="inlineStr">
         <is>
-          <t>抓取+搜索兜底均未找到，需人工核实</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1435,7 @@
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>2026.05.06</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H21" s="14" t="inlineStr">
@@ -1495,14 +1443,10 @@
           <t>https://www.ndss-symposium.org/ndss2027/</t>
         </is>
       </c>
-      <c r="I21" s="16" t="inlineStr">
-        <is>
-          <t>https://www.ndss-symposium.org/ndss2027/submissions/call-for-papers/</t>
-        </is>
-      </c>
+      <c r="I21" s="16" t="inlineStr"/>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K21" s="13" t="n"/>
@@ -1544,14 +1488,10 @@
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr"/>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>https://pldi26.sigplan.org/track/pldi-2026-PLDI-Workshops</t>
-        </is>
-      </c>
+      <c r="I22" s="9" t="inlineStr"/>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 Mon 24 Nov 2025 和会议年份 2027 对不上），需人工核实：https://pldi26.sigplan.org/track/pldi-2026-PLDI-Workshops</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1528,7 @@
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>2026.09.01</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H23" s="14" t="inlineStr">
@@ -1596,14 +1536,10 @@
           <t>https://aaai.org/conference/aaai/aaai-27/</t>
         </is>
       </c>
-      <c r="I23" s="16" t="inlineStr">
-        <is>
-          <t>https://aaai.org/conference/aaai/aaai-27/eaai-27-call/</t>
-        </is>
-      </c>
+      <c r="I23" s="16" t="inlineStr"/>
       <c r="J23" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K23" s="13" t="n"/>
@@ -1641,7 +1577,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>2026.07.06</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H24" s="14" t="inlineStr">
@@ -1649,14 +1585,10 @@
           <t>https://www.usenix.org/conference/fast27</t>
         </is>
       </c>
-      <c r="I24" s="16" t="inlineStr">
-        <is>
-          <t>https://iui.acm.org/2027/call-for-workshops/</t>
-        </is>
-      </c>
+      <c r="I24" s="16" t="inlineStr"/>
       <c r="J24" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K24" s="13" t="n"/>
@@ -1698,14 +1630,10 @@
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
-      <c r="I25" s="9" t="inlineStr">
-        <is>
-          <t>https://signalprocessingsociety.org/events/call-proposals-ssp-2027-2027-ieee-statistical-signal-processing-workshop</t>
-        </is>
-      </c>
+      <c r="I25" s="9" t="inlineStr"/>
       <c r="J25" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 27 November 2024 和会议年份 2027 对不上），需人工核实：https://signalprocessingsociety.org/events/call-proposals-ssp-2027-2027-ieee-statistical-signal-processing-workshop</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -1742,18 +1670,14 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H26" s="12" t="inlineStr"/>
-      <c r="I26" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I26" s="16" t="inlineStr"/>
       <c r="J26" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K26" s="13" t="n"/>
@@ -1795,14 +1719,10 @@
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
-      <c r="I27" s="9" t="inlineStr">
-        <is>
-          <t>https://conf.researchr.org/track/ase-2025/ase-2025-workshops</t>
-        </is>
-      </c>
+      <c r="I27" s="9" t="inlineStr"/>
       <c r="J27" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 April 25, 2025 和会议年份 2027 对不上），需人工核实：https://conf.researchr.org/track/ase-2025/ase-2025-workshops</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1811,7 @@
       </c>
       <c r="G29" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H29" s="14" t="inlineStr">
@@ -1899,14 +1819,10 @@
           <t>https://www.siam.org/conferences-events/siam-conferences/soda27/</t>
         </is>
       </c>
-      <c r="I29" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I29" s="16" t="inlineStr"/>
       <c r="J29" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K29" s="13" t="n"/>
@@ -1944,18 +1860,14 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H30" s="12" t="inlineStr"/>
-      <c r="I30" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I30" s="16" t="inlineStr"/>
       <c r="J30" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K30" s="13" t="n"/>
@@ -1993,18 +1905,14 @@
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H31" s="12" t="inlineStr"/>
-      <c r="I31" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I31" s="16" t="inlineStr"/>
       <c r="J31" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K31" s="13" t="n"/>
@@ -2053,7 +1961,7 @@
       <c r="I32" s="0" t="inlineStr"/>
       <c r="J32" s="0" t="inlineStr">
         <is>
-          <t>抓取+搜索兜底均未找到，需人工核实</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -2090,7 +1998,7 @@
       </c>
       <c r="G33" s="11" t="inlineStr">
         <is>
-          <t>2026.02.26</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H33" s="14" t="inlineStr">
@@ -2098,14 +2006,10 @@
           <t>https://kdd2027.kdd.org/</t>
         </is>
       </c>
-      <c r="I33" s="16" t="inlineStr">
-        <is>
-          <t>https://kdd2026.kdd.org/call-for-workshop-proposals/</t>
-        </is>
-      </c>
+      <c r="I33" s="16" t="inlineStr"/>
       <c r="J33" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K33" s="13" t="n"/>
@@ -2151,14 +2055,10 @@
           <t>https://2027.sigmod.org/</t>
         </is>
       </c>
-      <c r="I34" s="9" t="inlineStr">
-        <is>
-          <t>https://2027.sigmod.org/calls_papers_important_dates.shtml</t>
-        </is>
-      </c>
+      <c r="I34" s="9" t="inlineStr"/>
       <c r="J34" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 October 21, 2011 和会议年份 2027 对不上），需人工核实：https://2027.sigmod.org/calls_papers_important_dates.shtml</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -2203,14 +2103,10 @@
           <t>https://www.usenix.org/conference/nsdi27</t>
         </is>
       </c>
-      <c r="I35" s="9" t="inlineStr">
-        <is>
-          <t>http://www.wikicfp.com/cfp/program?id=2239</t>
-        </is>
-      </c>
+      <c r="I35" s="9" t="inlineStr"/>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 October 12, 2023 和会议年份 2027 对不上），需人工核实：http://www.wikicfp.com/cfp/program?id=2239</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2143,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>2026.11.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H36" s="14" t="inlineStr">
@@ -2255,14 +2151,10 @@
           <t>https://www.vldb.org/2027/</t>
         </is>
       </c>
-      <c r="I36" s="16" t="inlineStr">
-        <is>
-          <t>https://mpc-deadlines.github.io/</t>
-        </is>
-      </c>
+      <c r="I36" s="16" t="inlineStr"/>
       <c r="J36" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K36" s="13" t="n"/>
@@ -2300,18 +2192,14 @@
       </c>
       <c r="G37" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H37" s="12" t="inlineStr"/>
-      <c r="I37" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I37" s="16" t="inlineStr"/>
       <c r="J37" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K37" s="13" t="n"/>
@@ -2401,18 +2289,14 @@
       </c>
       <c r="G39" s="11" t="inlineStr">
         <is>
-          <t>2026.03.02</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H39" s="12" t="inlineStr"/>
-      <c r="I39" s="16" t="inlineStr">
-        <is>
-          <t>http://www.wikicfp.com/cfp/program?id=374</t>
-        </is>
-      </c>
+      <c r="I39" s="16" t="inlineStr"/>
       <c r="J39" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K39" s="13" t="n"/>
@@ -2454,14 +2338,10 @@
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" s="9" t="inlineStr">
-        <is>
-          <t>https://focs.computer.org/2025/call-for-workshops/</t>
-        </is>
-      </c>
+      <c r="I40" s="9" t="inlineStr"/>
       <c r="J40" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 September 5, 2025 和会议年份 2027 对不上），需人工核实：https://focs.computer.org/2025/call-for-workshops/</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -2498,18 +2378,14 @@
       </c>
       <c r="G41" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H41" s="12" t="inlineStr"/>
-      <c r="I41" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I41" s="16" t="inlineStr"/>
       <c r="J41" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K41" s="13" t="n"/>
@@ -2603,14 +2479,10 @@
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="9" t="inlineStr">
-        <is>
-          <t>https://sg.ieeevis.org/year/2025/info/call-participation/workshops</t>
-        </is>
-      </c>
+      <c r="I43" s="9" t="inlineStr"/>
       <c r="J43" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 August 1, 2025 和会议年份 2027 对不上），需人工核实：https://sg.ieeevis.org/year/2025/info/call-participation/workshops</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2519,7 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H44" s="14" t="inlineStr">
@@ -2655,14 +2527,10 @@
           <t>https://ieeevr.org/2027/</t>
         </is>
       </c>
-      <c r="I44" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I44" s="16" t="inlineStr"/>
       <c r="J44" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K44" s="13" t="n"/>
@@ -2700,18 +2568,14 @@
       </c>
       <c r="G45" s="11" t="inlineStr">
         <is>
-          <t>2026.06.01</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H45" s="12" t="inlineStr"/>
-      <c r="I45" s="16" t="inlineStr">
-        <is>
-          <t>https://www.isanet.org/Conferences/ISA2027/Call</t>
-        </is>
-      </c>
+      <c r="I45" s="16" t="inlineStr"/>
       <c r="J45" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K45" s="13" t="n"/>
@@ -2756,7 +2620,7 @@
       <c r="I46" s="0" t="inlineStr"/>
       <c r="J46" s="0" t="inlineStr">
         <is>
-          <t>抓取+搜索兜底均未找到，需人工核实</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -2793,18 +2657,14 @@
       </c>
       <c r="G47" s="11" t="inlineStr">
         <is>
-          <t>2026.06.06</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H47" s="12" t="inlineStr"/>
-      <c r="I47" s="16" t="inlineStr">
-        <is>
-          <t>https://neurips.cc/Conferences/2026/CallForWorkshops</t>
-        </is>
-      </c>
+      <c r="I47" s="16" t="inlineStr"/>
       <c r="J47" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K47" s="13" t="n"/>
@@ -2842,7 +2702,7 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H48" s="14" t="inlineStr">
@@ -2850,14 +2710,10 @@
           <t>https://2027.aclweb.org/</t>
         </is>
       </c>
-      <c r="I48" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I48" s="16" t="inlineStr"/>
       <c r="J48" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K48" s="13" t="n"/>
@@ -2899,14 +2755,10 @@
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr"/>
-      <c r="I49" s="9" t="inlineStr">
-        <is>
-          <t>https://zplatform.ai/ai-event/cvpr-2027/</t>
-        </is>
-      </c>
+      <c r="I49" s="9" t="inlineStr"/>
       <c r="J49" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 November 7, 2025 和会议年份 2027 对不上），需人工核实：https://zplatform.ai/ai-event/cvpr-2027/</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -2947,14 +2799,10 @@
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr"/>
-      <c r="I50" s="9" t="inlineStr">
-        <is>
-          <t>https://iccv.thecvf.com/Conferences/2025/CallForWorkshops</t>
-        </is>
-      </c>
+      <c r="I50" s="9" t="inlineStr"/>
       <c r="J50" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 Mar 13, 2025 和会议年份 2027 对不上），需人工核实：https://iccv.thecvf.com/Conferences/2025/CallForWorkshops</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -2991,18 +2839,14 @@
       </c>
       <c r="G51" s="11" t="inlineStr">
         <is>
-          <t>2026.09.28</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H51" s="12" t="inlineStr"/>
-      <c r="I51" s="16" t="inlineStr">
-        <is>
-          <t>https://chi2027.acm.org/authors/workshops/</t>
-        </is>
-      </c>
+      <c r="I51" s="16" t="inlineStr"/>
       <c r="J51" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K51" s="13" t="n"/>
@@ -3040,18 +2884,14 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>2026.02.06</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H52" s="12" t="inlineStr"/>
-      <c r="I52" s="16" t="inlineStr">
-        <is>
-          <t>https://2026.ijcai.org/ijcai-ecai-2026-call-for-workshop-proposals/</t>
-        </is>
-      </c>
+      <c r="I52" s="16" t="inlineStr"/>
       <c r="J52" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K52" s="13" t="n"/>
@@ -3089,18 +2929,14 @@
       </c>
       <c r="G53" s="11" t="inlineStr">
         <is>
-          <t>2026.04.10</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H53" s="12" t="inlineStr"/>
-      <c r="I53" s="16" t="inlineStr">
-        <is>
-          <t>https://cscw.acm.org/2026/workshops.html</t>
-        </is>
-      </c>
+      <c r="I53" s="16" t="inlineStr"/>
       <c r="J53" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K53" s="13" t="n"/>
@@ -3138,18 +2974,14 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>2026.07.06</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H54" s="12" t="inlineStr"/>
-      <c r="I54" s="16" t="inlineStr">
-        <is>
-          <t>https://iui.acm.org/2027/call-for-workshops/</t>
-        </is>
-      </c>
+      <c r="I54" s="16" t="inlineStr"/>
       <c r="J54" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K54" s="13" t="n"/>
@@ -3191,14 +3023,10 @@
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr"/>
-      <c r="I55" s="9" t="inlineStr">
-        <is>
-          <t>https://www.ubicomp.org/ubicomp-iswc-2025/workshop-proposals/</t>
-        </is>
-      </c>
+      <c r="I55" s="9" t="inlineStr"/>
       <c r="J55" s="0" t="inlineStr">
         <is>
-          <t>抓到疑似过期页面（页面日期 2025-05-03 和会议年份 2027 对不上），需人工核实：https://www.ubicomp.org/ubicomp-iswc-2025/workshop-proposals/</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -3235,18 +3063,14 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>2026.05.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H56" s="12" t="inlineStr"/>
-      <c r="I56" s="16" t="inlineStr">
-        <is>
-          <t>https://uist.acm.org/2026/cfp/</t>
-        </is>
-      </c>
+      <c r="I56" s="16" t="inlineStr"/>
       <c r="J56" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K56" s="13" t="n"/>
@@ -3284,7 +3108,7 @@
       </c>
       <c r="G57" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H57" s="14" t="inlineStr">
@@ -3292,14 +3116,10 @@
           <t>https://acmweb2027.org/</t>
         </is>
       </c>
-      <c r="I57" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I57" s="16" t="inlineStr"/>
       <c r="J57" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K57" s="13" t="n"/>
@@ -3337,18 +3157,14 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H58" s="12" t="inlineStr"/>
-      <c r="I58" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I58" s="16" t="inlineStr"/>
       <c r="J58" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K58" s="13" t="n"/>
@@ -3386,18 +3202,14 @@
       </c>
       <c r="G59" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H59" s="12" t="inlineStr"/>
-      <c r="I59" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I59" s="16" t="inlineStr"/>
       <c r="J59" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K59" s="13" t="n"/>
@@ -3435,18 +3247,14 @@
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>2026.02.13</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H60" s="12" t="inlineStr"/>
-      <c r="I60" s="16" t="inlineStr">
-        <is>
-          <t>https://icml.cc/Conferences/2026/CallForWorkshops</t>
-        </is>
-      </c>
+      <c r="I60" s="16" t="inlineStr"/>
       <c r="J60" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K60" s="13" t="n"/>
@@ -3495,7 +3303,7 @@
       <c r="I61" s="0" t="inlineStr"/>
       <c r="J61" s="0" t="inlineStr">
         <is>
-          <t>抓取+搜索兜底均未找到，需人工核实</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3340,7 @@
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>2026.09.04</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H62" s="14" t="inlineStr">
@@ -3540,14 +3348,10 @@
           <t>https://www.vlsisymposium.org/</t>
         </is>
       </c>
-      <c r="I62" s="16" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I62" s="16" t="inlineStr"/>
       <c r="J62" s="11" t="inlineStr">
         <is>
-          <t>extracted via search fallback（搜索兜底抽取，未核实页面是否确属该会议，需要人工审核）</t>
+          <t>需要人工核实官网（未配置搜索API做兜底）</t>
         </is>
       </c>
       <c r="K62" s="13" t="n"/>
@@ -3656,7 +3460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3741,974 +3545,1946 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>PPoPP</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>2026.07.24</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>FSE/ESEC</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>2027.03.05</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>ICDE</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>2026.05.19</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>MICRO</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>2026.09.28</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>SC</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>2026.08.28</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>EuroSys</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>2026.08.21</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>MobiCom</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>INFOCOM</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>2026.11.04</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>EUROCRYPT</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>2026.09.17</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>CRYPTO</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>2026.07.26</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>NDSS</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>2026.05.06</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>AAAI</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>2026.09.01</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>FAST</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>2026.07.06</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>OOPSLA</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>SODA</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>DAC</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>FM</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>SIGKDD</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>2026.02.26</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>VLDB</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>2026.11.04</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>STOC</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>CAV</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>2026.03.02</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>LICS</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>VR</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="0" t="inlineStr">
         <is>
           <t>ISSTA</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>2026.06.01</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t>NeurIPS</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>2026.06.06</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="0" t="inlineStr">
         <is>
           <t>ACL</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="0" t="inlineStr">
         <is>
           <t>ACM MM</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>2026.09.28</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="0" t="inlineStr">
         <is>
           <t>IJCAI</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>2026.02.06</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="0" t="inlineStr">
         <is>
           <t>CSCW</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>2026.04.10</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="0" t="inlineStr">
         <is>
           <t>SIGGRAPH</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>2026.07.06</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>UIST</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>2026.05.04</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t>WWW</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="0" t="inlineStr">
         <is>
           <t>RTSS</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="0" t="inlineStr">
         <is>
           <t>WINE</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>ICML</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>2026.02.13</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="0" t="inlineStr">
         <is>
           <t>VLSI</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>2026.09.04</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 12:50 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>PPoPP</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2026.07.24</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>FSE/ESEC</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2027.03.05</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ICDE</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2026.05.19</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>MICRO</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2026.09.28</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2026.08.28</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>EuroSys</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2026.08.21</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>MobiCom</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>INFOCOM</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2026.11.04</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>EUROCRYPT</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026.09.17</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026.07.26</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>NDSS</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026.05.06</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>AAAI</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2026.09.01</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>FAST</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026.07.06</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>OOPSLA</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SODA</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>DAC</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>FM</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SIGKDD</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2026.02.26</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>VLDB</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026.11.04</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>STOC</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>CAV</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2026.03.02</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>LICS</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>VR</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ISSTA</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2026.06.01</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>NeurIPS</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2026.06.06</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ACL</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ACM MM</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2026.09.28</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>IJCAI</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2026.02.06</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>CSCW</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2026.04.10</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>SIGGRAPH</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2026.07.06</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>UIST</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2026.05.04</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>WWW</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>RTSS</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>WINE</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ICML</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2026.02.13</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>VLSI</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2026.09.04</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:06 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix CHI deadline reverted to TBD by a transient fetch failure on last run
</commit_message>
<xml_diff>
--- a/data/Conferences.xlsx
+++ b/data/Conferences.xlsx
@@ -549,7 +549,11 @@
           <t>https://ppopp27.sigplan.org/</t>
         </is>
       </c>
-      <c r="I2" s="9" t="inlineStr"/>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>https://popl27.sigplan.org/track/POPL-2027-workshops-and-co-located-events</t>
+        </is>
+      </c>
       <c r="J2" s="7" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -598,7 +602,11 @@
           <t>https://conf.researchr.org/home/fse-2027</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr"/>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/fse-2027</t>
+        </is>
+      </c>
       <c r="J3" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -646,7 +654,11 @@
           <t>https://icde2027.github.io/</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr"/>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>https://icde2027.github.io/</t>
+        </is>
+      </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -738,7 +750,11 @@
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>https://chi2027.acm.org/authors/workshops/</t>
+        </is>
+      </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -782,7 +798,11 @@
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>https://sc26.supercomputing.org/all-dates-deadlines/</t>
+        </is>
+      </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -966,7 +986,11 @@
           <t>https://2027.eurosys.org/</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr"/>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>https://2027.eurosys.org/cfp.html</t>
+        </is>
+      </c>
       <c r="J11" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1010,7 +1034,11 @@
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>https://www.sigcomm.org/news</t>
+        </is>
+      </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1058,7 +1086,11 @@
           <t>https://www.sigmobile.org/mobicom/2027/</t>
         </is>
       </c>
-      <c r="I13" s="9" t="inlineStr"/>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J13" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1106,7 +1138,11 @@
           <t>https://infocom2027.ieee-infocom.org/</t>
         </is>
       </c>
-      <c r="I14" s="9" t="inlineStr"/>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>https://mpc-deadlines.github.io/</t>
+        </is>
+      </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1198,7 +1234,11 @@
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="9" t="inlineStr"/>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>http://www.wikicfp.com/cfp/program?id=399</t>
+        </is>
+      </c>
       <c r="J16" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1246,7 +1286,11 @@
           <t>https://eurocrypt.iacr.org/2027/</t>
         </is>
       </c>
-      <c r="I17" s="9" t="inlineStr"/>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>https://eurocrypt.iacr.org/2027/callforpapers.php</t>
+        </is>
+      </c>
       <c r="J17" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1294,7 +1338,11 @@
           <t>https://sp2027.ieee-security.org/index.html</t>
         </is>
       </c>
-      <c r="I18" s="9" t="inlineStr"/>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>https://signalprocessingsociety.org/events/call-proposals-ssp-2027-2027-ieee-statistical-signal-processing-workshop</t>
+        </is>
+      </c>
       <c r="J18" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1338,7 +1386,11 @@
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr"/>
-      <c r="I19" s="9" t="inlineStr"/>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>https://www.iacr.org/events/eventsbysubmission.php4</t>
+        </is>
+      </c>
       <c r="J19" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1434,7 +1486,11 @@
           <t>https://www.ndss-symposium.org/ndss2027/</t>
         </is>
       </c>
-      <c r="I21" s="9" t="inlineStr"/>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ndss-symposium.org/ndss2027/submissions/call-for-papers/</t>
+        </is>
+      </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1478,7 +1534,11 @@
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr"/>
-      <c r="I22" s="9" t="inlineStr"/>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>https://pldi26.sigplan.org/track/pldi-2026-PLDI-Workshops</t>
+        </is>
+      </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1526,7 +1586,11 @@
           <t>https://aaai.org/conference/aaai/aaai-27/</t>
         </is>
       </c>
-      <c r="I23" s="9" t="inlineStr"/>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>https://aaai.org/conference/aaai/aaai-27/eaai-27-call/</t>
+        </is>
+      </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1574,7 +1638,11 @@
           <t>https://www.usenix.org/conference/fast27</t>
         </is>
       </c>
-      <c r="I24" s="9" t="inlineStr"/>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>https://iui.acm.org/2027/call-for-workshops/</t>
+        </is>
+      </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1618,7 +1686,11 @@
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
-      <c r="I25" s="9" t="inlineStr"/>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>https://signalprocessingsociety.org/events/call-proposals-ssp-2027-2027-ieee-statistical-signal-processing-workshop</t>
+        </is>
+      </c>
       <c r="J25" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1662,7 +1734,11 @@
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="9" t="inlineStr"/>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J26" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1706,7 +1782,11 @@
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
-      <c r="I27" s="9" t="inlineStr"/>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/track/ase-2025/ase-2025-workshops</t>
+        </is>
+      </c>
       <c r="J27" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1806,7 +1886,11 @@
           <t>https://www.siam.org/conferences-events/siam-conferences/soda27/</t>
         </is>
       </c>
-      <c r="I29" s="9" t="inlineStr"/>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1850,7 +1934,11 @@
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
-      <c r="I30" s="9" t="inlineStr"/>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J30" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1894,7 +1982,11 @@
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="9" t="inlineStr"/>
+      <c r="I31" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J31" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1990,7 +2082,11 @@
           <t>https://kdd2027.kdd.org/</t>
         </is>
       </c>
-      <c r="I33" s="9" t="inlineStr"/>
+      <c r="I33" s="9" t="inlineStr">
+        <is>
+          <t>https://kdd2026.kdd.org/call-for-workshop-proposals/</t>
+        </is>
+      </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2038,7 +2134,11 @@
           <t>https://2027.sigmod.org/</t>
         </is>
       </c>
-      <c r="I34" s="9" t="inlineStr"/>
+      <c r="I34" s="9" t="inlineStr">
+        <is>
+          <t>https://2027.sigmod.org/calls_papers_important_dates.shtml</t>
+        </is>
+      </c>
       <c r="J34" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2086,7 +2186,11 @@
           <t>https://www.usenix.org/conference/nsdi27</t>
         </is>
       </c>
-      <c r="I35" s="9" t="inlineStr"/>
+      <c r="I35" s="9" t="inlineStr">
+        <is>
+          <t>http://www.wikicfp.com/cfp/program?id=2239</t>
+        </is>
+      </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2134,7 +2238,11 @@
           <t>https://www.vldb.org/2027/</t>
         </is>
       </c>
-      <c r="I36" s="9" t="inlineStr"/>
+      <c r="I36" s="9" t="inlineStr">
+        <is>
+          <t>https://mpc-deadlines.github.io/</t>
+        </is>
+      </c>
       <c r="J36" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2178,7 +2286,11 @@
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" s="9" t="inlineStr"/>
+      <c r="I37" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J37" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2218,7 +2330,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026.09.28</t>
         </is>
       </c>
       <c r="H38" s="14" t="inlineStr">
@@ -2226,10 +2338,14 @@
           <t>https://chi2027.acm.org/</t>
         </is>
       </c>
-      <c r="I38" s="16" t="inlineStr"/>
+      <c r="I38" s="16" t="inlineStr">
+        <is>
+          <t>https://chi2027.acm.org/authors/workshops/</t>
+        </is>
+      </c>
       <c r="J38" s="11" t="inlineStr">
         <is>
-          <t>需要人工核实官网（未配置搜索API做兜底）</t>
+          <t>extracted from official site</t>
         </is>
       </c>
       <c r="K38" s="13" t="n"/>
@@ -2271,7 +2387,11 @@
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="9" t="inlineStr"/>
+      <c r="I39" s="9" t="inlineStr">
+        <is>
+          <t>http://www.wikicfp.com/cfp/program?id=374</t>
+        </is>
+      </c>
       <c r="J39" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2315,7 +2435,11 @@
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" s="9" t="inlineStr"/>
+      <c r="I40" s="9" t="inlineStr">
+        <is>
+          <t>https://focs.computer.org/2025/call-for-workshops/</t>
+        </is>
+      </c>
       <c r="J40" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2359,7 +2483,11 @@
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="9" t="inlineStr"/>
+      <c r="I41" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J41" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2455,7 +2583,11 @@
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="9" t="inlineStr"/>
+      <c r="I43" s="9" t="inlineStr">
+        <is>
+          <t>https://sg.ieeevis.org/year/2025/info/call-participation/workshops</t>
+        </is>
+      </c>
       <c r="J43" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2503,7 +2635,11 @@
           <t>https://ieeevr.org/2027/</t>
         </is>
       </c>
-      <c r="I44" s="9" t="inlineStr"/>
+      <c r="I44" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J44" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2547,7 +2683,11 @@
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="9" t="inlineStr"/>
+      <c r="I45" s="9" t="inlineStr">
+        <is>
+          <t>https://www.isanet.org/Conferences/ISA2027/Call</t>
+        </is>
+      </c>
       <c r="J45" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2635,7 +2775,11 @@
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="9" t="inlineStr"/>
+      <c r="I47" s="9" t="inlineStr">
+        <is>
+          <t>https://neurips.cc/Conferences/2026/CallForWorkshops</t>
+        </is>
+      </c>
       <c r="J47" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2683,7 +2827,11 @@
           <t>https://2027.aclweb.org/</t>
         </is>
       </c>
-      <c r="I48" s="9" t="inlineStr"/>
+      <c r="I48" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J48" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2727,7 +2875,11 @@
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr"/>
-      <c r="I49" s="9" t="inlineStr"/>
+      <c r="I49" s="9" t="inlineStr">
+        <is>
+          <t>https://zplatform.ai/ai-event/cvpr-2027/</t>
+        </is>
+      </c>
       <c r="J49" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2771,7 +2923,11 @@
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr"/>
-      <c r="I50" s="9" t="inlineStr"/>
+      <c r="I50" s="9" t="inlineStr">
+        <is>
+          <t>https://iccv.thecvf.com/Conferences/2025/CallForWorkshops</t>
+        </is>
+      </c>
       <c r="J50" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2815,7 +2971,11 @@
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr"/>
-      <c r="I51" s="9" t="inlineStr"/>
+      <c r="I51" s="9" t="inlineStr">
+        <is>
+          <t>https://chi2027.acm.org/authors/workshops/</t>
+        </is>
+      </c>
       <c r="J51" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2859,7 +3019,11 @@
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr"/>
-      <c r="I52" s="9" t="inlineStr"/>
+      <c r="I52" s="9" t="inlineStr">
+        <is>
+          <t>https://2026.ijcai.org/ijcai-ecai-2026-call-for-workshop-proposals/</t>
+        </is>
+      </c>
       <c r="J52" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2903,7 +3067,11 @@
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr"/>
-      <c r="I53" s="9" t="inlineStr"/>
+      <c r="I53" s="9" t="inlineStr">
+        <is>
+          <t>https://cscw.acm.org/2026/workshops.html</t>
+        </is>
+      </c>
       <c r="J53" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2947,7 +3115,11 @@
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr"/>
-      <c r="I54" s="9" t="inlineStr"/>
+      <c r="I54" s="9" t="inlineStr">
+        <is>
+          <t>https://iui.acm.org/2027/call-for-workshops/</t>
+        </is>
+      </c>
       <c r="J54" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2991,7 +3163,11 @@
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr"/>
-      <c r="I55" s="9" t="inlineStr"/>
+      <c r="I55" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ubicomp.org/ubicomp-iswc-2025/workshop-proposals/</t>
+        </is>
+      </c>
       <c r="J55" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3035,7 +3211,11 @@
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr"/>
-      <c r="I56" s="9" t="inlineStr"/>
+      <c r="I56" s="9" t="inlineStr">
+        <is>
+          <t>https://uist.acm.org/2026/cfp/</t>
+        </is>
+      </c>
       <c r="J56" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3083,7 +3263,11 @@
           <t>https://acmweb2027.org/</t>
         </is>
       </c>
-      <c r="I57" s="9" t="inlineStr"/>
+      <c r="I57" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J57" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3127,7 +3311,11 @@
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr"/>
-      <c r="I58" s="9" t="inlineStr"/>
+      <c r="I58" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J58" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3171,7 +3359,11 @@
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr"/>
-      <c r="I59" s="9" t="inlineStr"/>
+      <c r="I59" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J59" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3215,7 +3407,11 @@
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr"/>
-      <c r="I60" s="9" t="inlineStr"/>
+      <c r="I60" s="9" t="inlineStr">
+        <is>
+          <t>https://icml.cc/Conferences/2026/CallForWorkshops</t>
+        </is>
+      </c>
       <c r="J60" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3311,7 +3507,11 @@
           <t>https://www.vlsisymposium.org/</t>
         </is>
       </c>
-      <c r="I62" s="9" t="inlineStr"/>
+      <c r="I62" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
+        </is>
+      </c>
       <c r="J62" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3422,7 +3622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5451,29 +5651,56 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="0" t="inlineStr">
         <is>
           <t>CHI</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
+      <c r="B76" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C76" s="0" t="inlineStr">
         <is>
           <t>2026.09.28</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
+      <c r="D76" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E76" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 14:07 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>2026.09.28</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2026-07-27 14:11 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix stale hyperlinks resurrecting old URLs after clear + save/reload
set_url() only cleared cell.value when the new url was empty, leaving
cell.hyperlink pointing at the old target. openpyxl reconstructs the
displayed value from a leftover hyperlink on save/reload even when
.value was set to "" in-process, so cleared workshopURL cells kept
showing stale (often wrong-conference) links from the earlier polluted
Brave Search run every time the file was reloaded. Now clears
cell.hyperlink and resets the font too. Re-ran the full pipeline and
verified only the 3 genuinely-confirmed rows have a workshopURL.
</commit_message>
<xml_diff>
--- a/data/Conferences.xlsx
+++ b/data/Conferences.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Arial"/>
       <sz val="11"/>
@@ -50,6 +50,7 @@
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font/>
   </fonts>
   <fills count="4">
     <fill>
@@ -87,7 +88,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -137,6 +138,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -549,11 +556,7 @@
           <t>https://ppopp27.sigplan.org/</t>
         </is>
       </c>
-      <c r="I2" s="9" t="inlineStr">
-        <is>
-          <t>https://popl27.sigplan.org/track/POPL-2027-workshops-and-co-located-events</t>
-        </is>
-      </c>
+      <c r="I2" s="19" t="inlineStr"/>
       <c r="J2" s="7" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -602,11 +605,7 @@
           <t>https://conf.researchr.org/home/fse-2027</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr">
-        <is>
-          <t>https://conf.researchr.org/home/fse-2027</t>
-        </is>
-      </c>
+      <c r="I3" s="19" t="inlineStr"/>
       <c r="J3" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -654,11 +653,7 @@
           <t>https://icde2027.github.io/</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
-        <is>
-          <t>https://icde2027.github.io/</t>
-        </is>
-      </c>
+      <c r="I4" s="19" t="inlineStr"/>
       <c r="J4" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -706,7 +701,7 @@
           <t>https://conf.researchr.org/home/hpca-2027</t>
         </is>
       </c>
-      <c r="I5" s="0" t="inlineStr"/>
+      <c r="I5" s="19" t="inlineStr"/>
       <c r="J5" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -749,12 +744,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr">
-        <is>
-          <t>https://chi2027.acm.org/authors/workshops/</t>
-        </is>
-      </c>
+      <c r="H6" s="18" t="inlineStr"/>
+      <c r="I6" s="19" t="inlineStr"/>
       <c r="J6" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -797,12 +788,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr">
-        <is>
-          <t>https://sc26.supercomputing.org/all-dates-deadlines/</t>
-        </is>
-      </c>
+      <c r="H7" s="18" t="inlineStr"/>
+      <c r="I7" s="19" t="inlineStr"/>
       <c r="J7" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -850,7 +837,7 @@
           <t>https://www.asplos-conference.org/asplos2027/cfp/</t>
         </is>
       </c>
-      <c r="I8" s="0" t="inlineStr"/>
+      <c r="I8" s="19" t="inlineStr"/>
       <c r="J8" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -893,8 +880,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="0" t="inlineStr"/>
+      <c r="H9" s="18" t="inlineStr"/>
+      <c r="I9" s="19" t="inlineStr"/>
       <c r="J9" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -937,8 +924,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="0" t="inlineStr"/>
+      <c r="H10" s="18" t="inlineStr"/>
+      <c r="I10" s="19" t="inlineStr"/>
       <c r="J10" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -986,11 +973,7 @@
           <t>https://2027.eurosys.org/</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>https://2027.eurosys.org/cfp.html</t>
-        </is>
-      </c>
+      <c r="I11" s="19" t="inlineStr"/>
       <c r="J11" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1033,12 +1016,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>https://www.sigcomm.org/news</t>
-        </is>
-      </c>
+      <c r="H12" s="18" t="inlineStr"/>
+      <c r="I12" s="19" t="inlineStr"/>
       <c r="J12" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1086,11 +1065,7 @@
           <t>https://www.sigmobile.org/mobicom/2027/</t>
         </is>
       </c>
-      <c r="I13" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1138,11 +1113,7 @@
           <t>https://infocom2027.ieee-infocom.org/</t>
         </is>
       </c>
-      <c r="I14" s="9" t="inlineStr">
-        <is>
-          <t>https://mpc-deadlines.github.io/</t>
-        </is>
-      </c>
+      <c r="I14" s="19" t="inlineStr"/>
       <c r="J14" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1190,7 +1161,7 @@
           <t>https://www.isscc.org/</t>
         </is>
       </c>
-      <c r="I15" s="0" t="inlineStr"/>
+      <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1233,12 +1204,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>http://www.wikicfp.com/cfp/program?id=399</t>
-        </is>
-      </c>
+      <c r="H16" s="18" t="inlineStr"/>
+      <c r="I16" s="19" t="inlineStr"/>
       <c r="J16" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1286,11 +1253,7 @@
           <t>https://eurocrypt.iacr.org/2027/</t>
         </is>
       </c>
-      <c r="I17" s="9" t="inlineStr">
-        <is>
-          <t>https://eurocrypt.iacr.org/2027/callforpapers.php</t>
-        </is>
-      </c>
+      <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1338,11 +1301,7 @@
           <t>https://sp2027.ieee-security.org/index.html</t>
         </is>
       </c>
-      <c r="I18" s="9" t="inlineStr">
-        <is>
-          <t>https://signalprocessingsociety.org/events/call-proposals-ssp-2027-2027-ieee-statistical-signal-processing-workshop</t>
-        </is>
-      </c>
+      <c r="I18" s="19" t="inlineStr"/>
       <c r="J18" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1385,12 +1344,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr"/>
-      <c r="I19" s="9" t="inlineStr">
-        <is>
-          <t>https://www.iacr.org/events/eventsbysubmission.php4</t>
-        </is>
-      </c>
+      <c r="H19" s="18" t="inlineStr"/>
+      <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1438,7 +1393,7 @@
           <t>https://www.usenix.org/conference/usenixsecurity27</t>
         </is>
       </c>
-      <c r="I20" s="0" t="inlineStr"/>
+      <c r="I20" s="19" t="inlineStr"/>
       <c r="J20" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1486,11 +1441,7 @@
           <t>https://www.ndss-symposium.org/ndss2027/</t>
         </is>
       </c>
-      <c r="I21" s="9" t="inlineStr">
-        <is>
-          <t>https://www.ndss-symposium.org/ndss2027/submissions/call-for-papers/</t>
-        </is>
-      </c>
+      <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1533,12 +1484,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr"/>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>https://pldi26.sigplan.org/track/pldi-2026-PLDI-Workshops</t>
-        </is>
-      </c>
+      <c r="H22" s="18" t="inlineStr"/>
+      <c r="I22" s="19" t="inlineStr"/>
       <c r="J22" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1586,11 +1533,7 @@
           <t>https://aaai.org/conference/aaai/aaai-27/</t>
         </is>
       </c>
-      <c r="I23" s="9" t="inlineStr">
-        <is>
-          <t>https://aaai.org/conference/aaai/aaai-27/eaai-27-call/</t>
-        </is>
-      </c>
+      <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1638,11 +1581,7 @@
           <t>https://www.usenix.org/conference/fast27</t>
         </is>
       </c>
-      <c r="I24" s="9" t="inlineStr">
-        <is>
-          <t>https://iui.acm.org/2027/call-for-workshops/</t>
-        </is>
-      </c>
+      <c r="I24" s="19" t="inlineStr"/>
       <c r="J24" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1685,12 +1624,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr"/>
-      <c r="I25" s="9" t="inlineStr">
-        <is>
-          <t>https://signalprocessingsociety.org/events/call-proposals-ssp-2027-2027-ieee-statistical-signal-processing-workshop</t>
-        </is>
-      </c>
+      <c r="H25" s="18" t="inlineStr"/>
+      <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1733,12 +1668,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="H26" s="18" t="inlineStr"/>
+      <c r="I26" s="19" t="inlineStr"/>
       <c r="J26" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1781,12 +1712,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr"/>
-      <c r="I27" s="9" t="inlineStr">
-        <is>
-          <t>https://conf.researchr.org/track/ase-2025/ase-2025-workshops</t>
-        </is>
-      </c>
+      <c r="H27" s="18" t="inlineStr"/>
+      <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1886,11 +1813,7 @@
           <t>https://www.siam.org/conferences-events/siam-conferences/soda27/</t>
         </is>
       </c>
-      <c r="I29" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I29" s="19" t="inlineStr"/>
       <c r="J29" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1933,12 +1856,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr"/>
-      <c r="I30" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="H30" s="18" t="inlineStr"/>
+      <c r="I30" s="19" t="inlineStr"/>
       <c r="J30" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -1981,12 +1900,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="H31" s="18" t="inlineStr"/>
+      <c r="I31" s="19" t="inlineStr"/>
       <c r="J31" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2034,7 +1949,7 @@
           <t>https://www.usenix.org/conference/osdi27</t>
         </is>
       </c>
-      <c r="I32" s="0" t="inlineStr"/>
+      <c r="I32" s="19" t="inlineStr"/>
       <c r="J32" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2082,11 +1997,7 @@
           <t>https://kdd2027.kdd.org/</t>
         </is>
       </c>
-      <c r="I33" s="9" t="inlineStr">
-        <is>
-          <t>https://kdd2026.kdd.org/call-for-workshop-proposals/</t>
-        </is>
-      </c>
+      <c r="I33" s="19" t="inlineStr"/>
       <c r="J33" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2134,11 +2045,7 @@
           <t>https://2027.sigmod.org/</t>
         </is>
       </c>
-      <c r="I34" s="9" t="inlineStr">
-        <is>
-          <t>https://2027.sigmod.org/calls_papers_important_dates.shtml</t>
-        </is>
-      </c>
+      <c r="I34" s="19" t="inlineStr"/>
       <c r="J34" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2186,11 +2093,7 @@
           <t>https://www.usenix.org/conference/nsdi27</t>
         </is>
       </c>
-      <c r="I35" s="9" t="inlineStr">
-        <is>
-          <t>http://www.wikicfp.com/cfp/program?id=2239</t>
-        </is>
-      </c>
+      <c r="I35" s="19" t="inlineStr"/>
       <c r="J35" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2238,11 +2141,7 @@
           <t>https://www.vldb.org/2027/</t>
         </is>
       </c>
-      <c r="I36" s="9" t="inlineStr">
-        <is>
-          <t>https://mpc-deadlines.github.io/</t>
-        </is>
-      </c>
+      <c r="I36" s="19" t="inlineStr"/>
       <c r="J36" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2285,12 +2184,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="H37" s="18" t="inlineStr"/>
+      <c r="I37" s="19" t="inlineStr"/>
       <c r="J37" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2298,57 +2193,56 @@
       </c>
     </row>
     <row r="38" ht="26.5" customHeight="1" s="8">
-      <c r="A38" s="11" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>交互</t>
         </is>
       </c>
-      <c r="B38" s="11" t="inlineStr">
+      <c r="B38" s="0" t="inlineStr">
         <is>
           <t>CHI</t>
         </is>
       </c>
-      <c r="C38" s="12" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>ACM Conference on Human Factors in Computing Systems</t>
         </is>
       </c>
-      <c r="D38" s="12" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>ACM</t>
         </is>
       </c>
-      <c r="E38" s="11" t="inlineStr">
+      <c r="E38" s="0" t="inlineStr">
         <is>
           <t>Pittsburgh, (PA), USA</t>
         </is>
       </c>
-      <c r="F38" s="11" t="inlineStr">
+      <c r="F38" s="0" t="inlineStr">
         <is>
           <t>05.10-05.14</t>
         </is>
       </c>
-      <c r="G38" s="11" t="inlineStr">
+      <c r="G38" s="0" t="inlineStr">
         <is>
           <t>2026.09.28</t>
         </is>
       </c>
-      <c r="H38" s="14" t="inlineStr">
+      <c r="H38" s="10" t="inlineStr">
         <is>
           <t>https://chi2027.acm.org/</t>
         </is>
       </c>
-      <c r="I38" s="16" t="inlineStr">
+      <c r="I38" s="9" t="inlineStr">
         <is>
           <t>https://chi2027.acm.org/authors/workshops/</t>
         </is>
       </c>
-      <c r="J38" s="11" t="inlineStr">
+      <c r="J38" s="0" t="inlineStr">
         <is>
           <t>extracted from official site</t>
         </is>
       </c>
-      <c r="K38" s="13" t="n"/>
     </row>
     <row r="39" ht="26.5" customHeight="1" s="8">
       <c r="A39" s="0" t="inlineStr">
@@ -2386,12 +2280,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="9" t="inlineStr">
-        <is>
-          <t>http://www.wikicfp.com/cfp/program?id=374</t>
-        </is>
-      </c>
+      <c r="H39" s="18" t="inlineStr"/>
+      <c r="I39" s="19" t="inlineStr"/>
       <c r="J39" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2434,12 +2324,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" s="9" t="inlineStr">
-        <is>
-          <t>https://focs.computer.org/2025/call-for-workshops/</t>
-        </is>
-      </c>
+      <c r="H40" s="18" t="inlineStr"/>
+      <c r="I40" s="19" t="inlineStr"/>
       <c r="J40" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2482,12 +2368,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="H41" s="18" t="inlineStr"/>
+      <c r="I41" s="19" t="inlineStr"/>
       <c r="J41" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2582,12 +2464,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="9" t="inlineStr">
-        <is>
-          <t>https://sg.ieeevis.org/year/2025/info/call-participation/workshops</t>
-        </is>
-      </c>
+      <c r="H43" s="18" t="inlineStr"/>
+      <c r="I43" s="19" t="inlineStr"/>
       <c r="J43" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2635,11 +2513,7 @@
           <t>https://ieeevr.org/2027/</t>
         </is>
       </c>
-      <c r="I44" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I44" s="19" t="inlineStr"/>
       <c r="J44" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2682,12 +2556,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="9" t="inlineStr">
-        <is>
-          <t>https://www.isanet.org/Conferences/ISA2027/Call</t>
-        </is>
-      </c>
+      <c r="H45" s="18" t="inlineStr"/>
+      <c r="I45" s="19" t="inlineStr"/>
       <c r="J45" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2730,8 +2600,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="0" t="inlineStr"/>
+      <c r="H46" s="18" t="inlineStr"/>
+      <c r="I46" s="19" t="inlineStr"/>
       <c r="J46" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2774,12 +2644,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="9" t="inlineStr">
-        <is>
-          <t>https://neurips.cc/Conferences/2026/CallForWorkshops</t>
-        </is>
-      </c>
+      <c r="H47" s="18" t="inlineStr"/>
+      <c r="I47" s="19" t="inlineStr"/>
       <c r="J47" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2827,11 +2693,7 @@
           <t>https://2027.aclweb.org/</t>
         </is>
       </c>
-      <c r="I48" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I48" s="19" t="inlineStr"/>
       <c r="J48" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2874,12 +2736,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H49" s="4" t="inlineStr"/>
-      <c r="I49" s="9" t="inlineStr">
-        <is>
-          <t>https://zplatform.ai/ai-event/cvpr-2027/</t>
-        </is>
-      </c>
+      <c r="H49" s="18" t="inlineStr"/>
+      <c r="I49" s="19" t="inlineStr"/>
       <c r="J49" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2922,12 +2780,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H50" s="4" t="inlineStr"/>
-      <c r="I50" s="9" t="inlineStr">
-        <is>
-          <t>https://iccv.thecvf.com/Conferences/2025/CallForWorkshops</t>
-        </is>
-      </c>
+      <c r="H50" s="18" t="inlineStr"/>
+      <c r="I50" s="19" t="inlineStr"/>
       <c r="J50" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -2970,12 +2824,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H51" s="4" t="inlineStr"/>
-      <c r="I51" s="9" t="inlineStr">
-        <is>
-          <t>https://chi2027.acm.org/authors/workshops/</t>
-        </is>
-      </c>
+      <c r="H51" s="18" t="inlineStr"/>
+      <c r="I51" s="19" t="inlineStr"/>
       <c r="J51" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3018,12 +2868,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H52" s="4" t="inlineStr"/>
-      <c r="I52" s="9" t="inlineStr">
-        <is>
-          <t>https://2026.ijcai.org/ijcai-ecai-2026-call-for-workshop-proposals/</t>
-        </is>
-      </c>
+      <c r="H52" s="18" t="inlineStr"/>
+      <c r="I52" s="19" t="inlineStr"/>
       <c r="J52" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3066,12 +2912,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H53" s="4" t="inlineStr"/>
-      <c r="I53" s="9" t="inlineStr">
-        <is>
-          <t>https://cscw.acm.org/2026/workshops.html</t>
-        </is>
-      </c>
+      <c r="H53" s="18" t="inlineStr"/>
+      <c r="I53" s="19" t="inlineStr"/>
       <c r="J53" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3114,12 +2956,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H54" s="4" t="inlineStr"/>
-      <c r="I54" s="9" t="inlineStr">
-        <is>
-          <t>https://iui.acm.org/2027/call-for-workshops/</t>
-        </is>
-      </c>
+      <c r="H54" s="18" t="inlineStr"/>
+      <c r="I54" s="19" t="inlineStr"/>
       <c r="J54" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3162,12 +3000,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H55" s="4" t="inlineStr"/>
-      <c r="I55" s="9" t="inlineStr">
-        <is>
-          <t>https://www.ubicomp.org/ubicomp-iswc-2025/workshop-proposals/</t>
-        </is>
-      </c>
+      <c r="H55" s="18" t="inlineStr"/>
+      <c r="I55" s="19" t="inlineStr"/>
       <c r="J55" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3210,12 +3044,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H56" s="4" t="inlineStr"/>
-      <c r="I56" s="9" t="inlineStr">
-        <is>
-          <t>https://uist.acm.org/2026/cfp/</t>
-        </is>
-      </c>
+      <c r="H56" s="18" t="inlineStr"/>
+      <c r="I56" s="19" t="inlineStr"/>
       <c r="J56" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3263,11 +3093,7 @@
           <t>https://acmweb2027.org/</t>
         </is>
       </c>
-      <c r="I57" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I57" s="19" t="inlineStr"/>
       <c r="J57" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3310,12 +3136,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H58" s="4" t="inlineStr"/>
-      <c r="I58" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="H58" s="18" t="inlineStr"/>
+      <c r="I58" s="19" t="inlineStr"/>
       <c r="J58" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3359,11 +3181,7 @@
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr"/>
-      <c r="I59" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I59" s="19" t="inlineStr"/>
       <c r="J59" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3406,12 +3224,8 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="H60" s="4" t="inlineStr"/>
-      <c r="I60" s="9" t="inlineStr">
-        <is>
-          <t>https://icml.cc/Conferences/2026/CallForWorkshops</t>
-        </is>
-      </c>
+      <c r="H60" s="18" t="inlineStr"/>
+      <c r="I60" s="19" t="inlineStr"/>
       <c r="J60" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3459,7 +3273,7 @@
           <t>https://ieee-iedm.org/</t>
         </is>
       </c>
-      <c r="I61" s="0" t="inlineStr"/>
+      <c r="I61" s="19" t="inlineStr"/>
       <c r="J61" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3507,11 +3321,7 @@
           <t>https://www.vlsisymposium.org/</t>
         </is>
       </c>
-      <c r="I62" s="9" t="inlineStr">
-        <is>
-          <t>https://www.aclweb.org/portal/content/joint-call-workshops-proposals-2027</t>
-        </is>
-      </c>
+      <c r="I62" s="19" t="inlineStr"/>
       <c r="J62" s="0" t="inlineStr">
         <is>
           <t>需要人工核实官网（未配置搜索API做兜底）</t>
@@ -3521,86 +3331,37 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId32"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.7480314960629921" right="0.7480314960629921" top="0.984251968503937" bottom="0.984251968503937" header="0.5118110236220472" footer="0.5118110236220472"/>
@@ -5678,27 +5439,27 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="0" t="inlineStr">
         <is>
           <t>CHI</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Workshop Deadline</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
+      <c r="B77" s="0" t="inlineStr">
+        <is>
+          <t>Workshop Deadline</t>
+        </is>
+      </c>
+      <c r="C77" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D77" s="0" t="inlineStr">
         <is>
           <t>2026.09.28</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E77" s="0" t="inlineStr">
         <is>
           <t>2026-07-27 14:11 UTC</t>
         </is>

</xml_diff>

<commit_message>
Add URL-pattern guessing and fix stale-location false positives
sync_base_info.py now guesses next-year URLs from ccfddl's previous-year
link pattern (e.g. pldi26.sigplan.org -> pldi27.sigplan.org) when ccfddl
hasn't added the target-year entry yet, verifying each guess actually
mentions the target year before trusting it. This recovered real 2027
info for SIGCOMM/PLDI/LICS/ACM MM/CoNEXT that was previously left TBD.

Also fixes a false positive where CoRL's location was silently filled in
from its still-current 2026 homepage (same domain every year) — location
extraction now requires the target year to appear near the match, same
as date extraction already did. Added day-first date parsing ('21-24
June 2027') and HTML entity decoding, both needed for the LICS fix.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Conferences.xlsx
+++ b/data/Conferences.xlsx
@@ -243,7 +243,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -451,6 +451,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1363,17 +1366,17 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Bangkok, Thailand</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>08.08-08.12</t>
         </is>
       </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>亚太</t>
         </is>
       </c>
       <c r="G12" s="14" t="inlineStr">
@@ -1391,7 +1394,11 @@
           <t>https://dblp.org/db/conf/sigcomm/</t>
         </is>
       </c>
-      <c r="J12" s="6" t="n"/>
+      <c r="J12" s="67" t="inlineStr">
+        <is>
+          <t>https://conferences.sigcomm.org/sigcomm/2027/</t>
+        </is>
+      </c>
       <c r="K12" s="60" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1599,7 +1606,7 @@
           <t>https://dblp.org/db/conf/ccs/</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="J16" s="67" t="inlineStr">
         <is>
           <t>https://www.sigsac.org/ccs/CCS2027/</t>
         </is>
@@ -1885,17 +1892,17 @@
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Atlanta, Georgia, USA</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>06.05-06.11</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>北美</t>
         </is>
       </c>
       <c r="G22" s="14" t="inlineStr">
@@ -1913,7 +1920,11 @@
           <t>https://dblp.org/db/conf/pldi/</t>
         </is>
       </c>
-      <c r="J22" s="6" t="n"/>
+      <c r="J22" s="67" t="inlineStr">
+        <is>
+          <t>https://pldi27.sigplan.org/</t>
+        </is>
+      </c>
       <c r="K22" s="60" t="inlineStr"/>
     </row>
     <row r="23" ht="28.5" customHeight="1" s="37">
@@ -2798,7 +2809,7 @@
           <t>https://dblp.org/db/conf/cav/</t>
         </is>
       </c>
-      <c r="J39" s="6" t="inlineStr">
+      <c r="J39" s="67" t="inlineStr">
         <is>
           <t>https://conferences.i-cav.org/2027/</t>
         </is>
@@ -2859,53 +2870,57 @@
       <c r="K40" s="60" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="13" t="inlineStr">
+      <c r="A41" s="38" t="inlineStr">
         <is>
           <t>理论</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
+      <c r="B41" s="38" t="inlineStr">
         <is>
           <t>LICS</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C41" s="39" t="inlineStr">
         <is>
           <t>ACM/IEEE Symposium on Logic in Computer Science</t>
         </is>
       </c>
-      <c r="D41" s="14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E41" s="15" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F41" s="14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G41" s="14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H41" s="16" t="inlineStr">
+      <c r="D41" s="40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E41" s="41" t="inlineStr">
+        <is>
+          <t>06.21-06.24</t>
+        </is>
+      </c>
+      <c r="F41" s="40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G41" s="40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H41" s="42" t="inlineStr">
         <is>
           <t>IEEE</t>
         </is>
       </c>
-      <c r="I41" s="17" t="inlineStr">
+      <c r="I41" s="43" t="inlineStr">
         <is>
           <t>https://dblp.org/db/conf/lics/</t>
         </is>
       </c>
-      <c r="J41" s="6" t="n"/>
-      <c r="K41" s="60" t="inlineStr"/>
+      <c r="J41" s="44" t="inlineStr">
+        <is>
+          <t>https://lics.siglog.org/lics27/</t>
+        </is>
+      </c>
+      <c r="K41" s="56" t="inlineStr"/>
     </row>
     <row r="42" ht="42.75" customHeight="1" s="37">
       <c r="A42" s="13" t="inlineStr">
@@ -3434,9 +3449,9 @@
           <t>https://dblp.org/db/conf/mm/</t>
         </is>
       </c>
-      <c r="J51" s="6" t="inlineStr">
-        <is>
-          <t>https://acmmm.org/</t>
+      <c r="J51" s="67" t="inlineStr">
+        <is>
+          <t>https://2027.acmmm.org/</t>
         </is>
       </c>
       <c r="K51" s="60" t="inlineStr"/>
@@ -3540,57 +3555,57 @@
       <c r="K53" s="60" t="inlineStr"/>
     </row>
     <row r="54" ht="42.75" customHeight="1" s="37">
-      <c r="A54" s="13" t="inlineStr">
+      <c r="A54" s="38" t="inlineStr">
         <is>
           <t>多媒体</t>
         </is>
       </c>
-      <c r="B54" s="13" t="inlineStr">
+      <c r="B54" s="38" t="inlineStr">
         <is>
           <t>SIGGRAPH</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C54" s="39" t="inlineStr">
         <is>
           <t>ACM Special Interest Group on Computer Graphics</t>
         </is>
       </c>
-      <c r="D54" s="14" t="inlineStr">
+      <c r="D54" s="40" t="inlineStr">
         <is>
           <t>Anaheim, USA</t>
         </is>
       </c>
-      <c r="E54" s="15" t="inlineStr">
-        <is>
-          <t>8.8-8.12</t>
-        </is>
-      </c>
-      <c r="F54" s="14" t="inlineStr">
+      <c r="E54" s="41" t="inlineStr">
+        <is>
+          <t>08.08-08.12</t>
+        </is>
+      </c>
+      <c r="F54" s="40" t="inlineStr">
         <is>
           <t>北美</t>
         </is>
       </c>
-      <c r="G54" s="14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H54" s="16" t="inlineStr">
+      <c r="G54" s="40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H54" s="42" t="inlineStr">
         <is>
           <t>ACM</t>
         </is>
       </c>
-      <c r="I54" s="17" t="inlineStr">
+      <c r="I54" s="43" t="inlineStr">
         <is>
           <t>https://dblp.org/db/conf/siggraph/</t>
         </is>
       </c>
-      <c r="J54" s="6" t="inlineStr">
+      <c r="J54" s="46" t="inlineStr">
         <is>
           <t>https://blog.siggraph.org/2025/01/inspiration-innovation-and-ice-cream-kristy-pron-to-lead-siggraph-2027.html/</t>
         </is>
       </c>
-      <c r="K54" s="60" t="inlineStr"/>
+      <c r="K54" s="56" t="inlineStr"/>
     </row>
     <row r="55" ht="28.5" customHeight="1" s="37">
       <c r="A55" s="13" t="inlineStr">
@@ -4382,57 +4397,57 @@
       <c r="K69" s="65" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="A70" s="52" t="inlineStr">
         <is>
           <t>光学</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B70" s="52" t="inlineStr">
         <is>
           <t>CLEO</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr">
+      <c r="C70" s="39" t="inlineStr">
         <is>
           <t>Conference on Lasers and Electro-Optics</t>
         </is>
       </c>
-      <c r="D70" s="14" t="inlineStr">
+      <c r="D70" s="40" t="inlineStr">
         <is>
           <t>Long Beach CA, USA</t>
         </is>
       </c>
-      <c r="E70" s="14" t="inlineStr">
-        <is>
-          <t>5.2-5.7</t>
-        </is>
-      </c>
-      <c r="F70" s="14" t="inlineStr">
+      <c r="E70" s="40" t="inlineStr">
+        <is>
+          <t>05.02-05.07</t>
+        </is>
+      </c>
+      <c r="F70" s="40" t="inlineStr">
         <is>
           <t>北美</t>
         </is>
       </c>
-      <c r="G70" s="0" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H70" s="3" t="inlineStr">
+      <c r="G70" s="73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H70" s="39" t="inlineStr">
         <is>
           <t>Optica/IEEE</t>
         </is>
       </c>
-      <c r="I70" s="6" t="inlineStr">
+      <c r="I70" s="46" t="inlineStr">
         <is>
           <t>https://ieeephotonics.org/</t>
         </is>
       </c>
-      <c r="J70" s="6" t="inlineStr">
+      <c r="J70" s="46" t="inlineStr">
         <is>
           <t>https://cleoconference.org/</t>
         </is>
       </c>
-      <c r="K70" s="65" t="inlineStr"/>
+      <c r="K70" s="63" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4505,7 +4520,7 @@
       </c>
       <c r="D72" s="14" t="inlineStr">
         <is>
-          <t>Austin , Texas</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E72" s="14" t="inlineStr">
@@ -4594,220 +4609,220 @@
       <c r="K73" s="65" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
+      <c r="A74" s="52" t="inlineStr">
         <is>
           <t>机器人</t>
         </is>
       </c>
-      <c r="B74" s="2" t="inlineStr">
+      <c r="B74" s="52" t="inlineStr">
         <is>
           <t>RSS</t>
         </is>
       </c>
-      <c r="C74" s="3" t="inlineStr">
+      <c r="C74" s="39" t="inlineStr">
         <is>
           <t>Robotics: Science and Systems</t>
         </is>
       </c>
-      <c r="D74" s="14" t="inlineStr">
+      <c r="D74" s="40" t="inlineStr">
         <is>
           <t>Athens, Greece</t>
         </is>
       </c>
-      <c r="E74" s="14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F74" s="14" t="inlineStr">
+      <c r="E74" s="40" t="inlineStr">
+        <is>
+          <t>07.06-07.11</t>
+        </is>
+      </c>
+      <c r="F74" s="40" t="inlineStr">
         <is>
           <t>欧洲</t>
         </is>
       </c>
-      <c r="G74" s="0" t="inlineStr">
+      <c r="G74" s="73" t="inlineStr">
         <is>
           <t>2026.04.23</t>
         </is>
       </c>
-      <c r="H74" s="3" t="inlineStr">
+      <c r="H74" s="39" t="inlineStr">
         <is>
           <t>RSS Foundation</t>
         </is>
       </c>
-      <c r="I74" s="29" t="inlineStr">
+      <c r="I74" s="55" t="inlineStr">
         <is>
           <t>https://roboticsconference.org/</t>
         </is>
       </c>
-      <c r="J74" s="6" t="inlineStr">
+      <c r="J74" s="46" t="inlineStr">
         <is>
           <t>https://roboticsconference.org/</t>
         </is>
       </c>
-      <c r="K74" s="72" t="inlineStr">
+      <c r="K74" s="64" t="inlineStr">
         <is>
           <t>https://roboticsconference.org/information/cfw/</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr">
+      <c r="A75" s="52" t="inlineStr">
         <is>
           <t>系统</t>
         </is>
       </c>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="B75" s="52" t="inlineStr">
         <is>
           <t>CGO</t>
         </is>
       </c>
-      <c r="C75" s="3" t="inlineStr">
+      <c r="C75" s="39" t="inlineStr">
         <is>
           <t>The International Symposium on Code Generation and Optimization</t>
         </is>
       </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>Salt Lake City, Utah</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>3.20-3.24</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
+      <c r="D75" s="53" t="inlineStr">
+        <is>
+          <t>Salt Lake City, Utah, USA</t>
+        </is>
+      </c>
+      <c r="E75" s="53" t="inlineStr">
+        <is>
+          <t>03.20-03.24</t>
+        </is>
+      </c>
+      <c r="F75" s="53" t="inlineStr">
         <is>
           <t>北美</t>
         </is>
       </c>
-      <c r="G75" s="0" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H75" s="3" t="inlineStr">
+      <c r="G75" s="73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H75" s="39" t="inlineStr">
         <is>
           <t>IEEE/ACM</t>
         </is>
       </c>
-      <c r="I75" s="6" t="inlineStr">
+      <c r="I75" s="46" t="inlineStr">
         <is>
           <t>https://dblp.org/db/conf/cgo/</t>
         </is>
       </c>
-      <c r="J75" s="6" t="inlineStr">
+      <c r="J75" s="46" t="inlineStr">
         <is>
           <t>https://2027.cgo.org/</t>
         </is>
       </c>
-      <c r="K75" s="65" t="inlineStr"/>
+      <c r="K75" s="63" t="inlineStr"/>
     </row>
     <row r="76" ht="29" customHeight="1" s="37">
-      <c r="A76" s="2" t="inlineStr">
+      <c r="A76" s="52" t="inlineStr">
         <is>
           <t>系统</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr">
+      <c r="B76" s="52" t="inlineStr">
         <is>
           <t>CC</t>
         </is>
       </c>
-      <c r="C76" s="3" t="inlineStr">
+      <c r="C76" s="39" t="inlineStr">
         <is>
           <t>International Conference on Compiler Construction</t>
         </is>
       </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>Salt Lake City, Utah</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>3.20-3.24</t>
-        </is>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
+      <c r="D76" s="53" t="inlineStr">
+        <is>
+          <t>Salt Lake City, Utah, USA</t>
+        </is>
+      </c>
+      <c r="E76" s="53" t="inlineStr">
+        <is>
+          <t>03.20-03.24</t>
+        </is>
+      </c>
+      <c r="F76" s="53" t="inlineStr">
         <is>
           <t>北美</t>
         </is>
       </c>
-      <c r="G76" s="0" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H76" s="3" t="inlineStr">
+      <c r="G76" s="73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H76" s="39" t="inlineStr">
         <is>
           <t>ACM</t>
         </is>
       </c>
-      <c r="I76" s="6" t="inlineStr">
+      <c r="I76" s="46" t="inlineStr">
         <is>
           <t>https://conf.researchr.org/home/CC-2026</t>
         </is>
       </c>
-      <c r="J76" s="6" t="inlineStr">
+      <c r="J76" s="46" t="inlineStr">
         <is>
           <t>https://conf.researchr.org/home/hpca-2027</t>
         </is>
       </c>
-      <c r="K76" s="65" t="inlineStr"/>
+      <c r="K76" s="63" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
+      <c r="A77" s="52" t="inlineStr">
         <is>
           <t>通信</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="B77" s="52" t="inlineStr">
         <is>
           <t>OFC</t>
         </is>
       </c>
-      <c r="C77" s="3" t="inlineStr">
+      <c r="C77" s="39" t="inlineStr">
         <is>
           <t>The Optical Fiber Communication Conference and Exhibition</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr">
+      <c r="D77" s="53" t="inlineStr">
         <is>
           <t>Los Angeles, California, USA</t>
         </is>
       </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>3.7-3.11</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
+      <c r="E77" s="53" t="inlineStr">
+        <is>
+          <t>03.07-03.11</t>
+        </is>
+      </c>
+      <c r="F77" s="53" t="inlineStr">
         <is>
           <t>北美</t>
         </is>
       </c>
-      <c r="G77" s="0" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H77" s="3" t="inlineStr">
+      <c r="G77" s="73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H77" s="39" t="inlineStr">
         <is>
           <t>IEEE/Optica</t>
         </is>
       </c>
-      <c r="I77" s="6" t="inlineStr">
+      <c r="I77" s="46" t="inlineStr">
         <is>
           <t>https://www.ofcconference.org/</t>
         </is>
       </c>
-      <c r="J77" s="6" t="inlineStr">
+      <c r="J77" s="46" t="inlineStr">
         <is>
           <t>https://www.ofcconference.org/</t>
         </is>
       </c>
-      <c r="K77" s="65" t="inlineStr"/>
+      <c r="K77" s="63" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5230,9 +5245,9 @@
           <t>https://dlnext.acm.org/conference/conext</t>
         </is>
       </c>
-      <c r="J85" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sigcomm.org/events/conext-conference</t>
+      <c r="J85" s="67" t="inlineStr">
+        <is>
+          <t>https://conferences.sigcomm.org/co-next/2027/#!/home</t>
         </is>
       </c>
       <c r="K85" s="65" t="inlineStr"/>
@@ -5645,131 +5660,135 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J85" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId146"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.7480314960629921" right="0.7480314960629921" top="0.984251968503937" bottom="0.984251968503937" header="0.5118110236220472" footer="0.5118110236220472"/>

</xml_diff>